<commit_message>
FOB nds SO upload & grouping BC 3.0 barang
</commit_message>
<xml_diff>
--- a/public/assets/template/template_upload_so.xlsx
+++ b/public/assets/template/template_upload_so.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -10,8 +10,8 @@
     <sheet name="UPLOAD PO" sheetId="23" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UPLOAD PO'!$A$1:$K$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'UPLOAD PO'!$G$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UPLOAD PO'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'UPLOAD PO'!$G$1:$L$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'UPLOAD PO'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>STYLE</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t>COLOR</t>
+  </si>
+  <si>
+    <t>FOB</t>
   </si>
   <si>
     <t>S</t>
@@ -89,15 +92,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="180" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="181" formatCode="[$-409]d\-mmm\-yy;@"/>
-    <numFmt numFmtId="182" formatCode="m/d/yyyy;@"/>
-    <numFmt numFmtId="183" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="181" formatCode="#,000_);[Red]\(#,000\)"/>
+    <numFmt numFmtId="182" formatCode="[$-409]d\-mmm\-yy;@"/>
+    <numFmt numFmtId="183" formatCode="m/d/yyyy;@"/>
+    <numFmt numFmtId="184" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="28">
     <font>
@@ -778,20 +782,24 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="182" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="181" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -803,11 +811,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="182" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="183" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="50" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="3" fillId="0" borderId="1" xfId="53" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="3" fillId="0" borderId="1" xfId="53" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="3" fillId="0" borderId="1" xfId="53" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -825,7 +836,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1148,7 +1159,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.2190476190476" style="1" customWidth="1"/>
@@ -1157,120 +1168,125 @@
     <col min="4" max="4" width="13.552380952381" style="1" customWidth="1"/>
     <col min="5" max="5" width="21.4380952380952" style="1" customWidth="1"/>
     <col min="6" max="7" width="24" style="1" customWidth="1"/>
-    <col min="8" max="11" width="9" style="1" customWidth="1"/>
-    <col min="12" max="17" width="9" style="1"/>
-    <col min="18" max="20" width="10.2857142857143" style="1"/>
-    <col min="21" max="16384" width="9" style="1"/>
+    <col min="8" max="8" width="9" style="3" customWidth="1"/>
+    <col min="9" max="12" width="9" style="1" customWidth="1"/>
+    <col min="13" max="18" width="9" style="1"/>
+    <col min="19" max="21" width="10.2857142857143" style="1"/>
+    <col min="22" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:11">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="1" customFormat="1" spans="1:12">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" ht="15" spans="1:11">
-      <c r="A2" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="7" t="s">
+    </row>
+    <row r="2" ht="15" spans="1:12">
+      <c r="A2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="C2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="10">
+      <c r="D2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="12">
         <v>46114</v>
       </c>
-      <c r="F2" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="11" t="s">
+      <c r="F2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="12">
+      <c r="G2" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="14"/>
+      <c r="I2" s="15">
         <v>425</v>
       </c>
-      <c r="I2" s="12">
+      <c r="J2" s="15">
         <v>376</v>
       </c>
-      <c r="J2" s="12">
+      <c r="K2" s="15">
         <v>362</v>
       </c>
-      <c r="K2" s="12">
+      <c r="L2" s="15">
         <v>217</v>
       </c>
     </row>
-    <row r="3" spans="11:11">
-      <c r="K3" s="13"/>
-    </row>
-    <row r="4" spans="11:11">
-      <c r="K4" s="14"/>
-    </row>
-    <row r="5" spans="11:11">
-      <c r="K5" s="13"/>
-    </row>
-    <row r="6" spans="11:11">
-      <c r="K6" s="14"/>
-    </row>
-    <row r="7" spans="11:11">
-      <c r="K7" s="13"/>
-    </row>
-    <row r="8" spans="11:11">
-      <c r="K8" s="14"/>
-    </row>
-    <row r="9" spans="11:11">
-      <c r="K9" s="13"/>
-    </row>
-    <row r="10" spans="11:11">
-      <c r="K10" s="14"/>
-    </row>
-    <row r="11" spans="11:11">
-      <c r="K11" s="13"/>
-    </row>
-    <row r="12" spans="11:11">
-      <c r="K12" s="14"/>
-    </row>
-    <row r="13" spans="11:11">
-      <c r="K13" s="13"/>
-    </row>
-    <row r="14" spans="11:11">
-      <c r="K14" s="14"/>
+    <row r="3" spans="1:12">
+      <c r="L3" s="16"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="L4" s="17"/>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="L5" s="16"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="L6" s="17"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="L7" s="16"/>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="L8" s="17"/>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="L9" s="16"/>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="L10" s="17"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="L11" s="16"/>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="L12" s="17"/>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="L13" s="16"/>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="L14" s="17"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:K2" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L2" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.196527777777778" right="0.0784722222222222" top="0.196527777777778" bottom="0.0784722222222222" header="0.0388888888888889" footer="0.0388888888888889"/>

</xml_diff>